<commit_message>
Update Master Report: 2026-03-20
</commit_message>
<xml_diff>
--- a/CR_News_Report_Master.xlsx
+++ b/CR_News_Report_Master.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
Update Master Report and High-Water Mark: 2026-03-20
</commit_message>
<xml_diff>
--- a/CR_News_Report_Master.xlsx
+++ b/CR_News_Report_Master.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J20"/>
+  <dimension ref="A1:J25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -483,45 +483,305 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>7 Best Food Processors and Choppers of 2026, Lab-Tested and Reviewed</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>https://www.consumerreports.org/appliances/food-processors-choppers/best-food-processors-of-the-year-a7878155198/</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Home Appliances</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Small Kitchen Appliances (Food Processors &amp; Choppers)</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Breville, Cuisinart, KitchenAid, Braun, Ninja</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Consumer Reports evaluated and ranked the top 7 food processors and choppers for 2026. The review highlights top-performing models from Cuisinart, Breville, KitchenAid, Braun, and Ninja based on lab tests for chopping, slicing, shredding, and noise levels.</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>The small kitchen appliance market for food processors is currently dominated by specialized brands like Cuisinart and Breville. Samsung and LG are not mentioned in this category, as they primarily focus on major home appliances rather than small countertop food preparation tools.</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Since Samsung does not compete in the food processor category, no direct competitive response is needed. However, the high importance placed on 'noise levels' and 'warranty length' in CR's scoring reflects consumer priorities that should be maintained in Samsung's core appliance categories.</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Best Drip Coffee Makers of 2026, Tested by Experts</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>https://www.consumerreports.org/appliances/coffee-makers/best-drip-coffee-makers-consumer-reports-tests-a1869713908/</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Home Appliances</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Kitchen Appliances (Coffee Makers)</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Bunn, Calphalon, Cuisinart, Haden, Hamilton Beach, Melitta</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Consumer Reports released its 2026 rankings for drip coffee makers, testing over 150 models. Top recommendations were categorized by type: traditional drip (Bunn, Calphalon, Cuisinart, Haden, Hamilton Beach), grind-and-brew (Cuisinart, Melitta), and self-serve (Cuisinart). Evaluation criteria included brew performance (temperature and contact time), ease of use, and owner satisfaction.</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Cuisinart emerged as a dominant brand across multiple sub-categories, earning high marks for both technical performance and owner satisfaction. Reliability and the ability to maintain optimal brewing temperatures (195°F-205°F) remain the primary differentiators for 'Recommended' status.</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>As Samsung does not currently compete in the coffee maker market, this report has no direct competitive impact. However, the high owner satisfaction scores for Cuisinart and Bunn highlight the importance of brand loyalty and reliability in the small kitchen appliance segment.</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>174,800 Frigidaire Gas Ranges Recalled Due to Burn Hazard</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>https://www.consumerreports.org/appliances/appliance-recalls/frigidaire-gas-ranges-recalled-burn-hazard-a1065367849/</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Home Appliances</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Cooktop, Wall-oven, Range</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Frigidaire, Electrolux</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Electrolux is recalling approximately 174,800 Frigidaire gas ranges due to a delayed ignition defect in the oven's bake burner, which poses a burn hazard. There have been 62 reports of malfunctions and 30 reported injuries. Consequently, Consumer Reports has withdrawn its recommendation for all nine Frigidaire gas range models currently in its ratings.</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>A major competitor (Frigidaire/Electrolux) has lost its 'Recommended' status across its entire gas range lineup in CR due to a significant safety recall. This creates a temporary vacuum in the 'Recommended' gas range category and potentially damages Frigidaire's brand reliability in the cooking segment.</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Samsung should capitalize on this competitor's safety issue by reinforcing the safety and reliability messaging of its own gas and electric range lineups. Marketing efforts could highlight Samsung's rigorous testing protocols to reassure consumers currently wary of gas range safety.</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>4 Best Whole-House Heat Pumps of 2026, Lab-Tested and Reviewed</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>https://www.consumerreports.org/appliances/heat-pumps/best-whole-house-heat-pumps-a1157154177/</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Home Appliances</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Air Conditioners (Heat Pumps)</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Frigidaire, Goodman, Trane, Lennox</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Consumer Reports tested and ranked the best whole-house ducted heat pumps for 2026. The top-performing models identified were the Frigidaire 3T, Goodman 3T R32, Trane 3T, and Lennox 3T, based on heating/cooling efficiency, noise levels, and brand reliability data.</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Traditional HVAC-focused brands (Frigidaire, Goodman, Trane, Lennox) continue to dominate the ducted heat pump category in Consumer Reports' rankings. Samsung and LG, despite their strength in ductless systems, were not mentioned or ranked in this specific report for whole-house ducted solutions.</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>While Samsung is a leader in the ductless mini-split market, the lack of presence in CR's ducted heat pump rankings—a segment now outselling gas furnaces—indicates a potential brand visibility or product testing gap in the North American whole-house replacement market.</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Best Deals on Headphones</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>https://www.consumerreports.org/electronics-computers/headphones/best-headphone-deals-a9608506602/</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Electronics</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Headphones</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Sonos, Apple, Google, Bose, JBL, Ozlo, Anker, Beats, Sony, Dyson, Sennheiser</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Consumer Reports identifies the best current deals on headphones and earbuds, evaluating models from major brands based on sound quality, noise cancellation, and battery life. Featured products include the Sony WF-1000XM5, Bose QuietComfort Ultra, and Apple AirPods 4.</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Samsung is completely absent from this list of recommended headphone deals, while key competitors like Apple, Sony, and Google are highlighted for their performance and value. Sony and Bose, in particular, are noted for top-tier noise cancellation and sound quality rankings.</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Given the absence of Galaxy Buds in this 'Best Deals' roundup, marketing should evaluate if current promotional pricing for Samsung audio products is being effectively communicated to reviewers or if performance gaps (real or perceived) are excluding them from CR's top-tier recommendations compared to Sony and Apple.</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
           <t>2026-03-19</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>Best Washers for $800 or Less</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>https://www.consumerreports.org/appliances/washing-machines/best-washers-for-800-dollars-or-less-a3982320572/</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>Appliances</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>Washing Machines</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>LG, Samsung, Electrolux, Maytag, Insignia</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t>컨슈머리포트는 800달러 이하의 가성비 세탁기 추천 목록을 발표하며, 봄철 신모델 출시로 인한 가격 상승 트렌드와 구매 적기를 분석했습니다. LG전자는 드럼, 교반식 통돌이, 고효율 통돌이 전 부문에서 다수의 모델이 '추천 제품(CR Recommended)'으로 선정되며 압도적인 성과를 거두었습니다. 반면 삼성전자는 고효율 통돌이 부문에서 1개 모델이 언급되었으나, 에너지 효율은 우수한 반면 사용자 만족도에서 최하위 점수를 기록하며 추천 목록에 포함되지 못했습니다.</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="H7" t="inlineStr">
         <is>
           <t>LG전자가 가성비 세탁기 시장의 주요 카테고리를 사실상 독점하며 브랜드 신뢰도와 성능 모두에서 경쟁 우위를 확고히 하고 있습니다. 삼성전자는 기술적 지표(에너지/물 효율)에서는 긍정적인 평가를 받았으나, 실사용자의 낮은 만족도와 신뢰도 문제가 브랜드 추천의 발목을 잡고 있어 이에 대한 품질 개선 및 이미지 회복이 시급한 상황입니다.</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="I7" t="inlineStr">
         <is>
           <t>- LG전자는 드럼(WM3400CW), 교반식(WT7005CW, WT7155CW), 고효율 통돌이(WT6100CW, WT8200CW) 등 전 부문에서 추천 제품(Top Pick)으로 선정됨.
 - 삼성전자 모델(WA52DG5500AV)은 에너지 효율, 물 효율, 진동 항목에서 최고 등급을 받았으나, 사용자 만족도(Owner Satisfaction)에서 최하위(Rock bottom) 점수를 기록함.
@@ -529,54 +789,54 @@
 - 달러 이하 보급형 시장에서 LG전자의 추천 모델 비중이 삼성전자를 압도하고 있으며, 삼성은 신뢰도 점수에서 경쟁사 대비 열세임.</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="J7" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
+    <row r="8">
+      <c r="A8" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>Best Deals on Vacuums</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>https://www.consumerreports.org/appliances/vacuum-cleaners/best-vacuum-deals-right-now-a5043984151/</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>Appliances</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>Vacuums</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>Samsung, LG, Black+Decker, Shark, Miele, Eufy, iRobot, GorFanty, Tineco, Kenmore, Bissell, Hoover, Dirt Devil, Bosch</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>Consumer Reports가 봄맞이 청소를 앞두고 스틱, 로봇, 업라이트, 캐니스터 등 다양한 진공청소기 카테고리의 할인 딜과 성능 평가 결과를 발표했습니다. Shark, Miele, Kenmore 등 주요 브랜드 제품들의 바닥 유형별 청소 성능, 반려동물 털 제거 능력, 사용자 편의성 등을 상세히 다루고 있습니다. 기사 본문은 주로 현재 할인 중인 모델들의 장단점을 분석하여 소비자들에게 구매 가이드를 제공하는 데 중점을 둡니다.</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="H8" t="inlineStr">
         <is>
           <t>기사 본문 설명에는 포함되지 않았으나, CR 공식 랭킹 데이터에서 'Samsung Bespoke AI Jet Ultra'가 83점으로 해당 카테고리 최고점 및 Top Pick으로 선정되었습니다. 이는 경쟁사인 LG CordZero(80점) 및 Miele, Bosch 등 프리미엄 브랜드를 제치고 성능 우위를 입증한 결과로, 프리미엄 무선 청소기 시장에서의 강력한 브랜드 위상을 보여줍니다.</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="I8" t="inlineStr">
         <is>
           <t>- Samsung Bespoke AI Jet Ultra 모델이 CR 평가 점수 83점으로 'TOP PICK' 및 'RECOMMENDED' 등급 획득.
 - Samsung Jet 85 모델이 79점을 기록하며 상위권 성능 유지 확인.
@@ -584,54 +844,54 @@
 - 기사 본문에서는 Shark, Miele, Kenmore 등 실질적인 할인 혜택이 있는 모델 위주로 상세 리뷰가 진행됨.</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="J8" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>9 Best Stick Vacuums of 2026, Lab-Tested and Reviewed</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>https://www.consumerreports.org/appliances/vacuum-cleaners/best-stick-vacuums-of-the-year-a1113185163/</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>Appliances</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>Stick Vacuums</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F9" t="inlineStr">
         <is>
           <t>Samsung, LG, Bosch, Miele, Shark</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="G9" t="inlineStr">
         <is>
           <t>컨슈머리포트가 2026년 최고의 스틱 청소기 9종을 선정하여 발표했습니다. 삼성전자의 '비스포크 AI 제트 울트라'는 강력한 흡입력과 긴 배터리 수명, 자동 먼지 비움 기능을 갖춘 충전 스테이션으로 높은 평가를 받으며 추천 제품(Top Pick)으로 선정되었습니다. LG전자의 '코드제로 올인원' 또한 카페트 청소 성능과 편의 기능에서 우수한 평가를 받았으나, 브랜드 신뢰도 면에서는 삼성이 더 높은 점수를 기록했습니다. 이 외에도 보쉬, 밀레, 샤크 등의 제품이 각 카테고리별 우수 모델로 이름을 올렸습니다.</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="H9" t="inlineStr">
         <is>
           <t>삼성전자의 프리미엄 스틱 청소기 라인업이 성능뿐만 아니라 브랜드 신뢰도 및 소유주 만족도 조사에서도 매우 우수한 성적을 거두고 있음을 확인했습니다. 특히 배터리 수명과 신뢰성 측면에서 경쟁사 대비 우위를 점하고 있어, 향후 북미 시장 내 프리미엄 가전 입지를 더욱 공고히 할 수 있을 것으로 분석됩니다.</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="I9" t="inlineStr">
         <is>
           <t>- 삼성 Bespoke AI Jet Ultra(VS90F40DMK/AA) 모델이 총점 83점으로 스틱 청소기 부문 'CR 추천 제품(Top Pick)' 선정.
 - 해당 모델은 바닥 및 반려동물 털 청소 성능에서 최고 등급을 받았으며, 테스트 모델 중 가장 긴 평균 작동 시간을 기록함.
@@ -639,54 +899,54 @@
 - 경쟁사인 LG CordZero A949KTMS는 총점 80점을 기록했으나, 브랜드 신뢰도 및 만족도 면에서는 중간 수준(Midlevel)에 머무름.</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="J9" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>2026-03-18</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>16 Best Washing Machines of 2026, Lab-Tested and Reviewed</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>https://www.consumerreports.org/appliances/washing-machines/best-washing-machines-of-the-year-a7327583525/</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>Appliances</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>Washing Machines</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>LG, Samsung, Miele, GE, Speed Queen, Electrolux, Amana, Frigidaire, Maytag, Whirlpool, Asko, Blomberg, Midea</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="G10" t="inlineStr">
         <is>
           <t>컨슈머리포트가 2026년 최고의 세탁기 16종을 선정하여 발표하였으며, LG전자가 드럼, 통돌이(교반식 및 고효율), 소형 드럼 등 거의 모든 주요 카테고리에서 추천 제품(Top Pick)을 휩쓸며 압도적인 성적을 거두었습니다. 삼성전자는 올인원 세탁건조기 부문에서 최고 점수를 기록했으나, 전체적인 추천 제품 리스트에서는 LG에 크게 밀리는 양상을 보였습니다. 특히 LG는 브랜드 신뢰도 조사에서도 드럼 및 고효율 통돌이 부문에서 가장 신뢰할 수 있는 브랜드로 꼽혔습니다.</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="H10" t="inlineStr">
         <is>
           <t>LG전자가 북미 세탁기 시장의 전 카테고리에서 성능과 신뢰성을 바탕으로 독보적인 우위를 점하고 있습니다. 삼성전자는 올인원 세탁건조기 시장에서 기술력을 인정받고 있으나, 주력 제품군인 일반 드럼 및 통돌이 세탁기 부문에서 LG의 '추천 제품' 독식을 견제할 수 있는 브랜드 신뢰도 회복 및 성능 차별화가 시급한 상황입니다.</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="I10" t="inlineStr">
         <is>
           <t>- LG전자가 드럼, 교반식 통돌이, 고효율 통돌이, 소형 드럼 등 4개 주요 부문에서 총 11개의 추천 제품(Top Pick)을 차지하며 시장 주도권 확인.
 - 삼성 올인원 세탁건조기(WD53DBA900HZ)는 해당 카테고리 최고 점수를 받았으나, 건조 성능 미흡 및 습도 센서 부재가 단점으로 지적됨.
@@ -694,54 +954,54 @@
 - Miele는 소형 드럼 세탁기 부문에서 높은 가격대에도 불구하고 우수한 성능과 사용자 만족도로 추천 제품에 다수 포함됨.</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="J10" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
+    <row r="11">
+      <c r="A11" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>How an Old-School Flip Phone Changed My Life</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>https://www.consumerreports.org/electronics-computers/cell-phones/pros-and-cons-of-using-a-flip-phone-a8412704280/</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D11" t="inlineStr">
         <is>
           <t>Electronics</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E11" t="inlineStr">
         <is>
           <t>Smartphones</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="F11" t="inlineStr">
         <is>
           <t>Samsung, Apple, Nokia, Mint Mobile, Cat, Light Phone, Bigme</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="G11" t="inlineStr">
         <is>
           <t>컨슈머리포트의 한 필자가 디지털 미니멀리즘을 실천하기 위해 아이폰 13 대신 노키아 2780 플립폰(덤폰)을 일주일간 사용한 경험을 공유했습니다. 플립폰 사용을 통해 스크린 타임을 하루 평균 3시간가량 줄이고 삶의 여유를 찾았으나, 앱 부재로 인한 차량 호출, 모바일 결제, 내비게이션 이용의 불편함과 낮은 카메라 성능 등의 한계가 명확히 드러났습니다. 필자는 스마트폰을 완전히 대체하기보다는 필요에 따라 스마트폰을 멀리하고 현재에 집중하기 위한 보조적 수단으로 플립폰 활용을 제안합니다.</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="H11" t="inlineStr">
         <is>
           <t>북미 시장 내 '디지털 디톡스'와 '덤폰(Dumb Phone)'에 대한 관심이 존재하지만, 실생활의 필수적인 앱 생태계와 고성능 카메라에 대한 의존도가 높아 스마트폰의 완전한 대체는 어려운 것으로 분석됩니다. 삼성전자는 갤럭시 S25 및 S24 시리즈가 CR 평가에서 최상위권을 유지하며 제품 경쟁력을 인정받고 있는 만큼, 압도적인 하드웨어 성능과 더불어 사용자의 효율적인 디지털 생활을 돕는 소프트웨어적 제어 기능을 강화하여 프리미엄 가치를 공고히 할 필요가 있습니다.</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="I11" t="inlineStr">
         <is>
           <t>- 삼성 갤럭시 S25 Ultra 및 S24 Ultra가 CR 스마트폰 평가에서 87점으로 공동 1위(Top Pick) 기록
 - 갤럭시 S25+ 모델 또한 86점으로 애플 아이폰 17 Pro Max와 함께 상위권 및 추천 제품 지위 유지
@@ -749,54 +1009,54 @@
 - 대다수 사용자는 스마트폰의 편리한 기능 때문에 완전한 기기 변경보다는 보조 기기 형태의 사용을 선호하는 경향을 보임</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="J11" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
+    <row r="12">
+      <c r="A12" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>Worst Vacuums We Tested—and What to Buy Instead</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>https://www.consumerreports.org/appliances/vacuum-cleaners/worst-vacuums-we-tested-and-what-to-buy-instead-a4744433209/</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>Appliances</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>Vacuums</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="F12" t="inlineStr">
         <is>
           <t>Samsung, LG, Shark, Kenmore, Eureka, Bissell, Dirt Devil, Ryobi, Eufy, Roborock, iRobot, Black+Decker</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="G12" t="inlineStr">
         <is>
           <t>Consumer Reports는 성능이 미흡한 '최악의 청소기' 목록과 이를 대체할 추천 모델을 발표했습니다. 무선 스틱 청소기 부문에서 Ryobi 모델의 대안으로 LG CordZero Q3가 추천되었으며, 카펫 청소 및 반려동물 털 제거 성능이 우수하다고 평가받았습니다. 한편, 별도 랭킹 데이터에 따르면 삼성전자의 Bespoke AI Jet Ultra가 83점으로 해당 카테고리에서 Top Pick으로 선정되었습니다. 전반적으로 저가형 모델의 흡입력 부족과 배출물 차단 실패가 주요 감점 요인으로 지적되었습니다.</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="H12" t="inlineStr">
         <is>
           <t>삼성전자의 Bespoke AI Jet Ultra가 최고점(83점)으로 Top Pick에 선정되어 프리미엄 무선 청소기 시장에서의 경쟁 우위를 확인했습니다. 경쟁사인 LG전자 또한 추천 모델 리스트에 포함되었으나, 삼성 모델이 점수 면에서 앞서고 있습니다. 소비자들이 저가형의 성능 한계를 인지하고 추천 모델로 이동하는 경향이 있으므로, 고성능 및 위생(Clean Emissions) 기능을 강조한 마케팅이 유효할 것으로 보입니다.</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="I12" t="inlineStr">
         <is>
           <t>- 삼성 Bespoke AI Jet Ultra 모델이 점수 83점으로 CR Recommended 및 Top Pick으로 선정됨.
 - 삼성 Jet 85 모델은 점수 79점으로 상위권에 랭크됨.
@@ -804,54 +1064,108 @@
 - 무선 스틱 청소기 평가에서 카펫 청소 성능, 반려동물 털 제거, 미세먼지 배출 차단 능력이 핵심 차별화 요소로 작용함.</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="J12" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>2026-03-16</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>ICYMI: Spring Yard Prep, Exclusive Member Savings, Apple's New MacBook Neo</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>https://www.consumerreports.org/home-garden/spring-yard-prep-exclusive-member-savings-apple-macbook-neo-a6548509942/</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Electronics &amp; Appliances</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Laptops, Microwaves</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Apple</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Consumer Reports의 최신 뉴스레터로, 애플이 599달러의 저가형 노트북인 '맥북 네오(MacBook Neo)'를 포함한 신규 라인업을 출시했다는 소식을 전하고 있습니다. 또한 주방 가전 및 수면 관련 제품에 대한 회원 전용 할인 혜택과 잔디 깎기 기계 관리법, 목재 스테인 내구성 테스트 결과 등을 다루었습니다. 현재 연구소에서는 카운터탑 전자레인지와 세탁 세제 등에 대한 최신 테스트가 진행 중임을 언급했습니다.</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>애플이 역대 최저가인 599달러 노트북을 출시하며 컴퓨팅 시장에서의 가격 진입장벽을 대폭 낮추었습니다. 이는 삼성전자의 갤럭시 북 등 보급형 노트북 라인업에 직접적인 경쟁 압박으로 작용할 수 있으며, CR이 전자레인지 부문의 최신 테스트를 진행 중이므로 향후 발표될 평가 결과에 대한 모니터링이 필요합니다.</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>- 애플, 역대 최저가인 599달러부터 시작하는 '맥북 네오(MacBook Neo)' 및 신규 맥북 에어/프로 라인업 발표
+- CR 연구소에서 카운터탑 전자레인지(Countertop Microwaves)에 대한 신규 테스트 및 평가 업데이트 진행 중
+- 월 17일까지 주방 가전 등 주요 카테고리 제품에 대해 최대 40%의 회원 전용 할인 혜택 제공</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-03-16</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
         <is>
           <t>Best Spring Cleaning Deals on Vacuums, Carpet Cleaners, and More</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>https://www.consumerreports.org/money/sales-promotions/best-spring-cleaning-deals-a6459257616/</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D14" t="inlineStr">
         <is>
           <t>Appliances</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E14" t="inlineStr">
         <is>
           <t>Vacuums, Air Purifiers, Carpet Cleaners</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="F14" t="inlineStr">
         <is>
           <t>Blueair, HoMedics, Dirt Devil, Hoover, Shark, iRobot, Dyson, Tineco, Levoit, Persil, Windex, Fabuloso, Method, Mrs. Meyers</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="G14" t="inlineStr">
         <is>
           <t>컨슈머리포트가 봄맞이 대청소 시즌을 맞아 진공청소기, 공기청정기, 카펫 클리너 등 주요 가전제품의 할인 및 추천 목록을 발표했습니다. iRobot Roomba Max 705가 로봇 청소기 중 최고 성능 제품으로 선정되었으며, Blueair의 공기청정기 시리즈가 높은 신뢰도와 성능을 바탕으로 추천 제품(Recommended)에 이름을 올렸습니다. Dyson V15 Detect와 Shark의 스틱 청소기 등 주요 경쟁사 제품들의 성능 테스트 결과와 할인 정보가 상세히 공유되었습니다.</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="H14" t="inlineStr">
         <is>
           <t>기사 내 삼성전자 제품에 대한 직접적인 언급은 없으나, 로봇 청소기 시장에서 iRobot이 압도적인 성능 평가를 받고 있으며 Dyson과 Shark가 프리미엄 및 실용성 시장을 주도하고 있음을 보여줍니다. 특히 공기청정기 분야에서 Blueair가 강력한 브랜드 신뢰도와 추천 등급을 확보하고 있어, 해당 카테고리 내 경쟁사들의 기술적 소구점과 프로모션 전략을 참고할 필요가 있습니다.</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="I14" t="inlineStr">
         <is>
           <t>- iRobot Roomba Max 705가 테스트 제품 중 최고 성능을 기록하며 100달러 할인된 가격으로 판매 중임.
 - Blueair 공기청정기 라인업(Mini Restful, 311i+ Max 등)이 CR 추천 제품으로 선정되었으며, 멤버십 대상 최대 40% 할인 코드 제공.
@@ -859,108 +1173,54 @@
 - Shark HydroVac Pro XL 및 Tineco Floor One S5가 스팀 및 세척 성능 부문에서 우수한 평가를 받음.</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="J14" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>2026-03-16</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>ICYMI: Spring Yard Prep, Exclusive Member Savings, Apple's New MacBook Neo</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>https://www.consumerreports.org/home-garden/spring-yard-prep-exclusive-member-savings-apple-macbook-neo-a6548509942/</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Electronics &amp; Appliances</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>Laptops, Microwaves</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>Apple</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>Consumer Reports의 최신 뉴스레터로, 애플이 599달러의 저가형 노트북인 '맥북 네오(MacBook Neo)'를 포함한 신규 라인업을 출시했다는 소식을 전하고 있습니다. 또한 주방 가전 및 수면 관련 제품에 대한 회원 전용 할인 혜택과 잔디 깎기 기계 관리법, 목재 스테인 내구성 테스트 결과 등을 다루었습니다. 현재 연구소에서는 카운터탑 전자레인지와 세탁 세제 등에 대한 최신 테스트가 진행 중임을 언급했습니다.</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>애플이 역대 최저가인 599달러 노트북을 출시하며 컴퓨팅 시장에서의 가격 진입장벽을 대폭 낮추었습니다. 이는 삼성전자의 갤럭시 북 등 보급형 노트북 라인업에 직접적인 경쟁 압박으로 작용할 수 있으며, CR이 전자레인지 부문의 최신 테스트를 진행 중이므로 향후 발표될 평가 결과에 대한 모니터링이 필요합니다.</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>- 애플, 역대 최저가인 599달러부터 시작하는 '맥북 네오(MacBook Neo)' 및 신규 맥북 에어/프로 라인업 발표
-- CR 연구소에서 카운터탑 전자레인지(Countertop Microwaves)에 대한 신규 테스트 및 평가 업데이트 진행 중
-- 월 17일까지 주방 가전 등 주요 카테고리 제품에 대해 최대 40%의 회원 전용 할인 혜택 제공</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
+    <row r="15">
+      <c r="A15" t="inlineStr">
         <is>
           <t>2026-03-13</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>5 Best Air Purifiers for Wildfire Smoke, According to Our Testing</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C15" t="inlineStr">
         <is>
           <t>https://www.consumerreports.org/appliances/air-purifiers/best-air-purifiers-for-wildfire-smoke-a1153295134/</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D15" t="inlineStr">
         <is>
           <t>Appliances</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="E15" t="inlineStr">
         <is>
           <t>Air Purifiers</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="F15" t="inlineStr">
         <is>
           <t>Coway, Blueair, AirDoctor, Winix, GermGuardian, Vissani, Honeywell</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="G15" t="inlineStr">
         <is>
           <t>컨슈머리포트는 산불 연기로 인한 대기 질 악화에 대비하여 미세 입자 제거 성능이 우수한 공기청정기 5종을 선정하여 발표했습니다. 테스트 결과 HEPA 필터를 장착하고 350평방피트 이상의 대형 공간을 커버하는 모델들이 연기 제거에 가장 효과적인 것으로 나타났습니다. 코웨이(Coway)의 Airmega ProX가 성능과 소음, 브랜드 신뢰도 면에서 최고 평가를 받았으며, 블루에어(Blueair)와 위닉스(Winix) 등의 제품이 추천 목록에 이름을 올렸습니다.</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="H15" t="inlineStr">
         <is>
           <t>북미 시장의 주요 구매 결정 요인 중 하나인 '산불 연기 대응 성능' 평가에서 삼성전자 제품이 추천 목록(Top 5)에 포함되지 않았습니다. 코웨이, 블루에어 등 공기청정기 전문 브랜드들이 성능뿐만 아니라 브랜드 신뢰도와 사용자 만족도에서도 높은 점수를 기록하며 시장 내 입지를 공고히 하고 있는 것으로 분석됩니다.</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="I15" t="inlineStr">
         <is>
           <t>- 컨슈머리포트 선정 산불 연기 제거 성능 우수 5대 공기청정기에 삼성 모델 미포함.
 - 코웨이 Airmega ProX가 대형 공간 정화 성능, 저소음, 브랜드 신뢰도에서 최고점(85점)을 받으며 Top Pick으로 선정됨.
@@ -969,54 +1229,54 @@
 - 추천된 모든 제품은 HEPA 필터를 탑재하고 350평방피트 이상의 대형 룸에 적합한 성능을 갖춘 것으로 확인됨.</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="J15" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
+    <row r="16">
+      <c r="A16" t="inlineStr">
         <is>
           <t>2026-03-12</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>Best Deals on Smart Home Devices</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C16" t="inlineStr">
         <is>
           <t>https://www.consumerreports.org/home-garden/smart-home/best-smart-home-deals-a3525616797/</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D16" t="inlineStr">
         <is>
           <t>Electronics</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="E16" t="inlineStr">
         <is>
           <t>Smart Home Devices</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="F16" t="inlineStr">
         <is>
           <t>TP-Link, Google, SimpliSafe, Amazon, Apple, Samsung</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
+      <c r="G16" t="inlineStr">
         <is>
           <t>컨슈머리포트가 보안 카메라, 스마트 플러그, 온도 조절기 등 주요 스마트 홈 기기의 최신 할인 정보와 테스트 결과를 발표했습니다. TP-Link의 Tapo 및 Kasa 라인업은 구독료 없는 AI 기능과 로컬 저장소 지원으로 높은 가성비를 인정받았으며, Google Nest 제품군은 우수한 비디오 품질과 보안성으로 추천되었습니다. 특히 다수의 추천 제품들이 삼성 SmartThings를 포함한 주요 스마트 홈 플랫폼과의 호환성을 주요 특징으로 내세우고 있습니다.</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="H16" t="inlineStr">
         <is>
           <t>삼성전자의 직접적인 하드웨어 제품은 언급되지 않았으나, TP-Link와 Google 등 주요 스마트 홈 기기 제조사들이 자사 제품의 핵심 경쟁력으로 'Samsung SmartThings' 호환성을 강조하고 있습니다. 이는 스마트 홈 생태계 내에서 SmartThings의 플랫폼 영향력이 견고함을 보여주며, 향후 Matter 표준 확산에 따른 기기 간 연결성 강화가 소비자 선택의 주요 기준이 될 것임을 시사합니다.</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
+      <c r="I16" t="inlineStr">
         <is>
           <t>- TP-Link Kasa Smart Wi-Fi Plug Slim EP25는 에너지 모니터링 기능을 제공하며 Samsung SmartThings를 포함한 4대 스마트 홈 시스템과 호환됨.
 - Google Nest Cam with Floodlight는 객체 감지 기능을 무료로 제공하며 Samsung SmartThings 앱 및 음성 제어를 지원함.
@@ -1024,54 +1284,54 @@
 - TP-Link Tapo 보안 카메라 시리즈는 구독료 없이 AI 감지 기능을 제공하며 높은 가성비로 추천됨.</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="J16" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
+    <row r="17">
+      <c r="A17" t="inlineStr">
         <is>
           <t>2026-03-11</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>Which iPhone Should You Buy?</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>https://www.consumerreports.org/electronics-computers/cell-phones/which-iphone-should-you-buy-a7028071026/</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D17" t="inlineStr">
         <is>
           <t>Electronics</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="E17" t="inlineStr">
         <is>
           <t>Smartphones</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="F17" t="inlineStr">
         <is>
           <t>Apple, Samsung</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
+      <c r="G17" t="inlineStr">
         <is>
           <t>컨슈머리포트가 애플의 최신 아이폰 17 라인업(17, 17e, Air, 17 Pro, 17 Pro Max)에 대한 구매 가이드를 발표했습니다. 각 모델별로 A19 칩셋을 통한 AI 기능 지원, 카메라 성능 차이, 배터리 수명 및 내구성 테스트 결과를 상세히 다루고 있습니다. 특히 새롭게 추가된 초슬림 모델인 '아이폰 Air'와 고성능 'Pro' 시리즈의 사양 및 가격대를 비교 분석했습니다.</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
+      <c r="H17" t="inlineStr">
         <is>
           <t>애플의 최신 아이폰 17 시리즈 출시 및 대대적인 홍보에도 불구하고, 컨슈머리포트의 종합 평가 점수에서는 삼성전자의 갤럭시 S25 울트라와 S24 울트라가 87점으로 공동 1위를 유지하며 아이폰 17 프로 맥스(86점)를 앞서고 있습니다. 이는 삼성전자의 플래그십 스마트폰이 하드웨어 성능과 사용자 경험 측면에서 여전히 시장 최고의 경쟁력을 확보하고 있음을 입증합니다.</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr">
+      <c r="I17" t="inlineStr">
         <is>
           <t>- 컨슈머리포트 스마트폰 부문 평가에서 삼성 갤럭시 S25 Ultra 및 S24 Ultra가 87점으로 전체 공동 1위 및 Top Pick 선정.
 - 애플의 최신 플래그십인 아이폰 17 Pro Max는 86점을 기록하여 삼성전자 상위 모델 대비 낮은 점수 획득.
@@ -1079,54 +1339,54 @@
 - 아이폰 17 시리즈는 전 모델 AI 기능 지원, 120Hz 주사율 확대, 기본 저장용량 증설(256GB) 등 하드웨어 상향 평준화가 진행됨.</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr">
+      <c r="J17" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
+    <row r="18">
+      <c r="A18" t="inlineStr">
         <is>
           <t>2026-03-10</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>What's the Best Mac Laptop or Desktop for You?</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C18" t="inlineStr">
         <is>
           <t>https://www.consumerreports.org/electronics-computers/computers/best-mac-desktop-or-laptop-for-you-a1085516654/</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="D18" t="inlineStr">
         <is>
           <t>Electronics</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="E18" t="inlineStr">
         <is>
           <t>Computing (Laptops, Desktops)</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="F18" t="inlineStr">
         <is>
           <t>Apple, MSI, HP, Acer, Asus, Intel</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
+      <c r="G18" t="inlineStr">
         <is>
           <t>애플이 아이폰 칩을 탑재한 599달러의 초저가형 '맥북 네오'를 포함하여 M5 칩셋 기반의 새로운 맥북 에어 및 프로 라인업을 발표했습니다. 신제품들은 AI 작업 성능이 대폭 향상되었고 WiFi 7을 지원하는 등 하드웨어 사양이 강화되었으나, 모델별로 100달러에서 최대 400달러까지 가격이 인상되었습니다. 컨슈머리포트는 맥북 프로, 에어, 맥 미니 등 애플의 주요 신규 라인업을 '추천 제품(Recommended)'으로 선정하며 높은 평가를 부여했습니다.</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
+      <c r="H18" t="inlineStr">
         <is>
           <t>애플이 저가형 시장(맥북 네오)부터 고성능 프리미엄 시장(M5 Max)까지 라인업을 촘촘히 재편하며 시장 점유율 확대를 꾀하고 있습니다. 특히 AI 성능 강화와 독자 생태계 확장은 삼성 갤럭시 북 시리즈에 위협 요소가 될 수 있으며, 애플의 가격 인상 정책이 시장 전체의 평균 판매 단가(ASP) 및 소비자 선택에 미칠 영향을 모니터링해야 합니다.</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr">
+      <c r="I18" t="inlineStr">
         <is>
           <t>- 애플, 아이폰 A18 Pro 칩을 탑재한 599달러 저가형 '맥북 네오' 출시로 보급형 시장 공략.
 - 신형 맥북 에어(M5) 및 맥북 프로(M5 Pro/Max) 라인업 공개 및 가격 인상(에어 100달러, 프로 16인치 모델 400달러 인상).
@@ -1134,54 +1394,54 @@
 - 컨슈머리포트 평가 결과, 맥북 프로(81점), 맥북 에어(76점), 아이맥(75점) 등 주요 신제품이 추천 제품(Recommended)으로 선정됨.</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr">
+      <c r="J18" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
+    <row r="19">
+      <c r="A19" t="inlineStr">
         <is>
           <t>2026-03-06</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B19" t="inlineStr">
         <is>
           <t>9 Best Desktop Computers of 2026, Tested by Our Experts</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C19" t="inlineStr">
         <is>
           <t>https://www.consumerreports.org/electronics-computers/computers/best-desktop-computers-of-the-year-a7188203360/</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D19" t="inlineStr">
         <is>
           <t>Computing</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="E19" t="inlineStr">
         <is>
           <t>Desktop Computers</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="F19" t="inlineStr">
         <is>
           <t>HP, Apple, Dell, Asus, MSI, Acer</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
+      <c r="G19" t="inlineStr">
         <is>
           <t>컨슈머리포트가 2026년 최고의 데스크탑 컴퓨터 9종을 선정하여 발표했습니다. 올인원, 미니 PC, 타워형의 세 가지 카테고리로 구분하여 성능, 신뢰도, 소비자 만족도를 평가했으며 HP, 애플, 델, 에이수스, MSI, 에이서 제품이 추천 목록에 올랐습니다. 특히 최신 인텔 Ultra, AMD Ryzen AI, 애플 M4 프로세서를 탑재하여 AI 기능을 강화한 모델들이 생산성 측면에서 높은 점수를 받았습니다.</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
+      <c r="H19" t="inlineStr">
         <is>
           <t>데스크탑 시장이 AI PC와 고성능 미니 PC 중심으로 재편되고 있는 가운데, 삼성전자의 제품은 단 한 모델도 추천 목록에 포함되지 못했습니다. 경쟁사들이 전문가용, 게이밍, 사무용 등 세부 시장에서 강력한 성능과 브랜드 신뢰도를 구축하고 있는 반면, 삼성전자의 데스크탑 라인업은 컨슈머리포트의 주요 평가 대상에서 소외되어 있어 브랜드 위상 제고가 시급해 보입니다.</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr">
+      <c r="I19" t="inlineStr">
         <is>
           <t>- 컨슈머리포트 선정 2026년 베스트 데스크탑 9종 목록에 삼성전자 제품 미포함
 - MSI Codex R2 Gaming Desktop이 86점으로 전체 최고점 기록
@@ -1190,54 +1450,54 @@
 - HP와 에이서는 게이밍 및 올인원 부문에서 긴 보증 기간(24~36개월)을 강점으로 내세워 추천됨</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr">
+      <c r="J19" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
+    <row r="20">
+      <c r="A20" t="inlineStr">
         <is>
           <t>2026-03-05</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B20" t="inlineStr">
         <is>
           <t>6 Best Robot Vacuums of 2026 for Pet Hair, Lab-Tested and Reviewed</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C20" t="inlineStr">
         <is>
           <t>https://www.consumerreports.org/appliances/vacuum-cleaners/best-robotic-vacuums-for-pet-hair-a6341573082/</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="D20" t="inlineStr">
         <is>
           <t>Appliances</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="E20" t="inlineStr">
         <is>
           <t>Robot Vacuums</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
+      <c r="F20" t="inlineStr">
         <is>
           <t>Samsung, LG, Dyson, Eufy, iRobot, Miele, Shark, Dreame, Eureka, Bosch</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
+      <c r="G20" t="inlineStr">
         <is>
           <t>컨슈머리포트가 반려동물 털 제거 성능이 우수한 2026년 최고의 로봇청소기 6종을 선정했습니다. 삼성전자의 Jet Bot VR7MD96514G 모델은 고가임에도 불구하고 강력한 흡입력과 테스트 제품 중 가장 뛰어난 물걸레 성능을 인정받아 추천 명단에 이름을 올렸습니다. 다이슨, 유피, 아이로봇, 드림, 유레카 등의 경쟁 모델들도 흡입 효율, 가성비, 내비게이션 성능 등을 바탕으로 함께 선정되었습니다.</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
+      <c r="H20" t="inlineStr">
         <is>
           <t>삼성전자의 로봇청소기는 특히 물걸레 성능 면에서 '테스트한 모든 제품 중 최고'라는 압도적인 평가를 받으며 프리미엄 가전으로서의 경쟁력을 입증했습니다. 또한 별도의 랭킹 데이터에서 Bespoke AI Jet Ultra 모델이 83점으로 Top Pick에 선정되는 등 주요 카테고리에서 상위권을 유지하고 있습니다. 다만 다이슨과 유피가 브랜드 신뢰도에서 강세를 보이고 있어, 성능 우위와 더불어 장기적인 신뢰도 관리가 필요할 것으로 보입니다.</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr">
+      <c r="I20" t="inlineStr">
         <is>
           <t>- 삼성 Jet Bot VR7MD96514G 모델이 반려동물 털 제거 및 물걸레 성능 우수로 'Best 6' 제품에 선정됨
 - 해당 모델의 물걸레 기능은 컨슈머리포트가 테스트한 모든 로봇청소기 겸용 모델 중 가장 우수하다고 명시됨
@@ -1246,54 +1506,54 @@
 - 다이슨은 신뢰도 면에서 매우 우수하나 사용자 만족도는 낮게 평가되었으며, 아이로봇은 파산 신청 상태이나 성능 면에서는 여전히 추천됨</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr">
+      <c r="J20" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
+    <row r="21">
+      <c r="A21" t="inlineStr">
         <is>
           <t>2026-03-04</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B21" t="inlineStr">
         <is>
           <t>8 Best Air Purifiers of 2026, Tested by Our Experts</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C21" t="inlineStr">
         <is>
           <t>https://www.consumerreports.org/appliances/air-purifiers/best-air-purifiers-of-the-year-a1197763201/</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="D21" t="inlineStr">
         <is>
           <t>Appliances</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="E21" t="inlineStr">
         <is>
           <t>Air Purifiers</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
+      <c r="F21" t="inlineStr">
         <is>
           <t>Coway, AirDoctor, Blueair, Honeywell, Vissani, GermGuardian</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr">
+      <c r="G21" t="inlineStr">
         <is>
           <t>컨슈머리포트가 2026년 공간 크기별 최고의 공기청정기 8종을 선정하여 발표했습니다. 평가 항목에는 미세먼지 및 연기 제거 성능, 소음 수준, 필터 교체비와 전기료를 합산한 연간 유지비용, 그리고 브랜드 신뢰도가 포함되었습니다. Coway Airmega ProX가 대형 공간용에서 최고점을 받았으며, Blueair와 Honeywell 제품들이 중소형 공간용 추천 제품으로 다수 이름을 올렸습니다.</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
+      <c r="H21" t="inlineStr">
         <is>
           <t>이번 추천 목록에 삼성전자 제품은 포함되지 않았으며, Coway와 Blueair가 성능과 신뢰도 면에서 시장을 주도하고 있는 것으로 나타났습니다. 특히 Coway는 대형 공간용 부문에서 독보적인 성능과 높은 브랜드 신뢰도를 기록하며 Top Pick으로 선정되었습니다. 경쟁사 LG 또한 이번 주요 순위권에는 언급되지 않았습니다.</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr">
+      <c r="I21" t="inlineStr">
         <is>
           <t>- 컨슈머리포트 2026년 공기청정기 부문 추천 제품 발표 (삼성 모델 미포함)
 - Coway Airmega ProX가 총점 85점으로 대형 공간용 부문 Top Pick 선정
@@ -1301,54 +1561,54 @@
 - 주요 평가 지표: 고속/저속 가동 시 입자 제거 효율, 소음, 연간 운영 비용(필터 및 전기료), 브랜드 신뢰도</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr">
+      <c r="J21" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
+    <row r="22">
+      <c r="A22" t="inlineStr">
         <is>
           <t>2026-03-04</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B22" t="inlineStr">
         <is>
           <t>Guide to Streaming Video Services</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C22" t="inlineStr">
         <is>
           <t>https://www.consumerreports.org/electronics-computers/streaming-media/guide-to-streaming-video-services-a4517732799/</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D22" t="inlineStr">
         <is>
           <t>Electronics</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="E22" t="inlineStr">
         <is>
           <t>TVs / Streaming Services</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
+      <c r="F22" t="inlineStr">
         <is>
           <t>Amazon, Apple, Disney, Hulu, Netflix, HBO Max, Paramount, Peacock, Sony, AMC, Google, Fubo, DirecTV</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr">
+      <c r="G22" t="inlineStr">
         <is>
           <t>본 기사는 넷플릭스, 디즈니+, 애플 TV+ 등 주요 스트리밍 서비스의 최신 요금제, 콘텐츠 특징 및 스포츠 중계권 현황을 상세히 가이드합니다. 최근 스트리밍 업계의 트렌드인 광고형 요금제 도입, 계정 공유 제한 정책, 그리고 라이브 TV 서비스의 가격 인상 및 번들 결합 상품 정보를 제공합니다. 또한 아마존과 디즈니의 NBA 중계권 확보 등 스포츠 콘텐츠 강화 움직임과 서비스 간 인수합병 소식을 다룹니다.</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr">
+      <c r="H22" t="inlineStr">
         <is>
           <t>삼성 스마트 TV(Tizen OS) 생태계 내에서 주요 스트리밍 앱의 접근성과 통합 검색 기능이 중요해지고 있습니다. 특히 스포츠 중계권이 여러 플랫폼으로 분산되고 서비스 간 번들링이 가속화됨에 따라, 소비자가 여러 서비스를 편리하게 전환하고 관리할 수 있는 인터페이스 제공이 하드웨어 경쟁력의 핵심 요소가 될 것으로 분석됩니다.</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr">
+      <c r="I22" t="inlineStr">
         <is>
           <t>- 넷플릭스, 디즈니+, 훌루 등 주요 서비스의 요금 인상 및 광고형 요금제 전면 도입.
 - 아마존, 디즈니, NBC유니버설의 NBA 중계권 확보 (2025/2026 시즌부터 11년간).
@@ -1357,54 +1617,54 @@
 - YouTube TV의 스포츠, 뉴스 등 장르별 세분화된 저가형 패키지 출시 계획 (2026년).</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr">
+      <c r="J22" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
+    <row r="23">
+      <c r="A23" t="inlineStr">
         <is>
           <t>2026-03-04</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B23" t="inlineStr">
         <is>
           <t>6 Live TV Streaming Services That Let You Cut Cable TV</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C23" t="inlineStr">
         <is>
           <t>https://www.consumerreports.org/electronics-computers/streaming-media/video-streaming-services-that-let-you-cut-cable-tv-a9076884300/</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D23" t="inlineStr">
         <is>
           <t>Electronics</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="E23" t="inlineStr">
         <is>
           <t>Streaming Services &amp; Devices</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
+      <c r="F23" t="inlineStr">
         <is>
           <t>DirecTV, Fubo, Hulu, Philo, Sling TV, YouTube, Google, Amazon, Apple, Roku, Nvidia</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr">
+      <c r="G23" t="inlineStr">
         <is>
           <t>케이블 TV를 대체할 수 있는 6가지 주요 라이브 TV 스트리밍 서비스(DirecTV, Fubo, Hulu + Live TV, Philo, Sling TV, YouTube TV)의 요금제와 채널 구성, 주요 특징을 비교 분석한 기사입니다. 각 서비스는 로컬 방송 및 스포츠 채널 제공 여부, 클라우드 DVR 저장 용량 등에서 차이를 보이며 최근 가격 인상 추세를 보이고 있습니다. 또한, 이러한 서비스를 이용하기에 적합한 4K 스트리밍 기기로 Roku, Amazon, Google, Apple, Nvidia의 제품들을 추천하고 있습니다.</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr">
+      <c r="H23" t="inlineStr">
         <is>
           <t>삼성 스마트 TV의 Tizen OS 플랫폼은 기사에서 언급된 Roku, Apple TV, Google TV Streamer 등 외부 스트리밍 기기들과 콘텐츠 허브 주도권을 두고 경쟁 관계에 있습니다. 소비자 리포트가 추천한 'Top Pick' 기기들이 삼성 TV의 내장 플랫폼 기능을 대체할 수 있는 만큼, 삼성 TV 사용자들의 이탈을 막기 위해 주요 스트리밍 서비스와의 파트너십 강화 및 내장 앱의 사용성 개선이 중요합니다.</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr">
+      <c r="I23" t="inlineStr">
         <is>
           <t>- Consumer Reports는 Roku Ultra(2024), Amazon Fire TV Cube(3rd Gen), Google TV Streamer(4K), Apple TV 4K, Nvidia Shield TV Pro를 스트리밍 기기 부문 'Top Pick'으로 선정함.
 - YouTube TV($72/월), Hulu + Live TV($90~100/월), Fubo($85~110/월) 등 주요 라이브 스트리밍 서비스의 요금 인상 및 채널 패키지 변경 사항이 보고됨.
@@ -1412,108 +1672,108 @@
 - 주요 스트리밍 기기들은 4K 해상도 지원, 멀티뷰 기능, 무제한 클라우드 DVR 등을 핵심 경쟁력으로 내세우고 있음.</t>
         </is>
       </c>
-      <c r="J18" t="inlineStr">
+      <c r="J23" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
+    <row r="24">
+      <c r="A24" t="inlineStr">
         <is>
           <t>2026-03-03</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B24" t="inlineStr">
         <is>
           <t>3 Reasons to Choose a Hand Mixer Over a Stand Mixer</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C24" t="inlineStr">
         <is>
           <t>https://www.consumerreports.org/appliances/mixers/reasons-to-choose-a-hand-mixer-over-a-stand-mixer-a5008456414/</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="D24" t="inlineStr">
         <is>
           <t>Appliances</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="E24" t="inlineStr">
         <is>
           <t>Mixers</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
+      <c r="F24" t="inlineStr">
         <is>
           <t>KitchenAid, Breville, Cuisinart, Toastmaster, Braun, Pioneer Woman, Beautiful by Drew Barrymore, Hamilton Beach</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr">
+      <c r="G24" t="inlineStr">
         <is>
           <t>컨슈머리포트는 가벼운 반죽 조리, 공간 절약, 저렴한 비용을 이유로 스탠드 믹서보다 핸드 믹서가 효율적일 수 있음을 설명하며 구매 가이드를 제공함. 주요 성능 테스트 항목으로는 혼합 성능, 소음, 편의성 등이 포함되었으며 세척 관리의 중요성을 강조함. Braun, Breville, Cuisinart, KitchenAid의 특정 모델들이 우수한 평가를 받으며 추천 제품으로 선정됨.</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr">
+      <c r="H24" t="inlineStr">
         <is>
           <t>해당 기사는 소형 주방 가전인 핸드 믹서를 다루고 있으며, 삼성전자가 주력으로 하는 가전 카테고리에 해당하지 않아 직접적인 비즈니스 영향은 미미함.</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr">
+      <c r="I24" t="inlineStr">
         <is>
           <t>- 컨슈머리포트의 핸드 믹서 부문 성능 평가 결과 및 추천 제품 리스트 발표.
 - Braun, Breville, Cuisinart, KitchenAid 제품이 'Top Pick' 및 추천 모델로 선정됨.
 - 삼성전자 및 LG전자 관련 언급이나 해당 카테고리 내 경쟁 제품은 포함되지 않음.</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr">
+      <c r="J24" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
+    <row r="25">
+      <c r="A25" t="inlineStr">
         <is>
           <t>2026-03-03</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B25" t="inlineStr">
         <is>
           <t>Best TV Deals Right Now</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C25" t="inlineStr">
         <is>
           <t>https://www.consumerreports.org/electronics-computers/tvs/best-tv-deals-right-now-a7570913441/</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="D25" t="inlineStr">
         <is>
           <t>Electronics</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="E25" t="inlineStr">
         <is>
           <t>TVs, Soundbars, Streaming Devices</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
+      <c r="F25" t="inlineStr">
         <is>
           <t>Samsung, LG, Sony, TCL, Hisense, Insignia, Roku, Amazon</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr">
+      <c r="G25" t="inlineStr">
         <is>
           <t>컨슈머리포트는 3월 스포츠 시즌을 앞두고 현재 할인 중인 주요 TV 모델들의 성능 평가와 추천 순위를 발표했습니다. 삼성전자의 QD-OLED 및 OLED TV 모델들은 화질과 사운드 부문에서 최고 점수인 91점을 기록하며 'Top Pick'으로 선정되었으나, 보급형인 Crystal UHD 라인업은 HDR 성능 미흡이 지적되었습니다. LG전자의 C5 OLED 시리즈 역시 삼성과 동일한 최고점을 기록하며 강력한 경쟁 모델로 평가받았습니다.</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr">
+      <c r="H25" t="inlineStr">
         <is>
           <t>삼성전자의 프리미엄 라인업(QD-OLED, OLED)은 화질과 사운드에서 업계 최고 수준의 경쟁력을 입증하며 추천 제품 상단을 점유하고 있습니다. 하지만 보급형 시장에서는 HDR 성능 부족이 지속적으로 언급되고 있으며, TCL과 Hisense 등 중국 브랜드들이 미니 LED 기술을 앞세워 가성비 시장을 공략하고 있어 이에 대한 대응이 필요합니다.</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr">
+      <c r="I25" t="inlineStr">
         <is>
           <t>- 삼성 QD-OLED(QN77S90C) 및 OLED(QN65S84FA) 모델이 화질 및 HDR 성능에서 최고 수준의 평가를 받으며 CR 추천 제품(Top Pick)으로 선정됨.
 - 보급형 Crystal UHD 라인업(UN507900F 등)은 일반 화질은 양호하나 HDR 표현력 부족이 주요 단점으로 반복 지적됨.
@@ -1521,7 +1781,7 @@
 - 삼성 9.1.4 채널 사운드바가 무선 돌비 애트모스 및 액티브 보이스 앰플리파이어 기능을 바탕으로 긍정적인 시장 기대를 얻고 있음.</t>
         </is>
       </c>
-      <c r="J20" t="inlineStr">
+      <c r="J25" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>

</xml_diff>

<commit_message>
Update Master Report and High-Water Mark: 2026-03-21
</commit_message>
<xml_diff>
--- a/CR_News_Report_Master.xlsx
+++ b/CR_News_Report_Master.xlsx
@@ -1369,12 +1369,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>AI Data Centers: Big Tech's Impact on Electric Bills, Water, and More</t>
+          <t>What to Expect for Amazon Prime Day 2026</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/data-centers/ai-data-centers-impact-on-electric-bills-water-and-more-a1040338678/</t>
+          <t>https://www.consumerreports.org/money/sales-promotions/amazon-prime-day-what-to-expect-a9781954357/</t>
         </is>
       </c>
     </row>
@@ -1386,12 +1386,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>4 Best Toilet Brushes of 2026 From Our Evaluations</t>
+          <t>4 Best Whole-House Heat Pumps of 2026, Lab-Tested and Reviewed</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/home-garden/toilets/best-toilet-brushes-a6509646029/</t>
+          <t>https://www.consumerreports.org/appliances/heat-pumps/best-whole-house-heat-pumps-a1157154177/</t>
         </is>
       </c>
     </row>
@@ -1403,12 +1403,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Best TV Brands of 2026</t>
+          <t>7 Best Food Processors and Choppers of 2026, Lab-Tested and Reviewed</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/electronics-computers/tvs/best-tv-brands-a7582471181/</t>
+          <t>https://www.consumerreports.org/appliances/food-processors-choppers/best-food-processors-of-the-year-a7878155198/</t>
         </is>
       </c>
     </row>
@@ -1420,12 +1420,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Best Decking of 2026, Tested by Experts</t>
+          <t>Consumer Safety Agency Finalizes New Regulations on Water Beads and Infant Neck Floats</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/home-garden/decking/best-decking-materials-from-consumer-reports-tests-a6751297873/</t>
+          <t>https://www.consumerreports.org/babies-kids/toys/consumer-safety-agency-new-rules-water-beads-neck-floats-a2051187866/</t>
         </is>
       </c>
     </row>
@@ -1437,12 +1437,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Consumer Reports’ Used Car Checklist to Avoid Costly Repairs</t>
+          <t>Best Drip Coffee Makers of 2026, Tested by Experts</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/cars/how-to-inspect-a-used-car-a1377126659/</t>
+          <t>https://www.consumerreports.org/appliances/coffee-makers/best-drip-coffee-makers-consumer-reports-tests-a1869713908/</t>
         </is>
       </c>
     </row>
@@ -1454,12 +1454,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>11 Best Cordless Drills of 2026, Lab-Tested and Reviewed</t>
+          <t>174,800 Frigidaire Gas Ranges Recalled Due to Burn Hazard</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/home-garden/cordless-drills-impact-drivers/best-cordless-drills-of-the-year-a1168250583/</t>
+          <t>https://www.consumerreports.org/appliances/appliance-recalls/frigidaire-gas-ranges-recalled-burn-hazard-a1065367849/</t>
         </is>
       </c>
     </row>
@@ -1471,12 +1471,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Best Used Small Cars for Gas Mileage: Standout Picks From Consumer Reports' Fuel-Economy Tests</t>
+          <t>Best Deals on Headphones</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/cars/used-compact-cars-with-best-fuel-economy-a7463598571/</t>
+          <t>https://www.consumerreports.org/electronics-computers/headphones/best-headphone-deals-a9608506602/</t>
         </is>
       </c>
     </row>
@@ -1488,12 +1488,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>What to Expect for Amazon Prime Day 2026</t>
+          <t>AI Data Centers: Big Tech's Impact on Electric Bills, Water, and More</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/money/sales-promotions/amazon-prime-day-what-to-expect-a9781954357/</t>
+          <t>https://www.consumerreports.org/data-centers/ai-data-centers-impact-on-electric-bills-water-and-more-a1040338678/</t>
         </is>
       </c>
     </row>
@@ -1505,12 +1505,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Best Deals on Headphones</t>
+          <t>Best Used Small Cars for Gas Mileage: Standout Picks From Consumer Reports' Fuel-Economy Tests</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/electronics-computers/headphones/best-headphone-deals-a9608506602/</t>
+          <t>https://www.consumerreports.org/cars/used-compact-cars-with-best-fuel-economy-a7463598571/</t>
         </is>
       </c>
     </row>
@@ -1522,12 +1522,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>174,800 Frigidaire Gas Ranges Recalled Due to Burn Hazard</t>
+          <t>Consumer Reports’ Used Car Checklist to Avoid Costly Repairs</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/appliances/appliance-recalls/frigidaire-gas-ranges-recalled-burn-hazard-a1065367849/</t>
+          <t>https://www.consumerreports.org/cars/how-to-inspect-a-used-car-a1377126659/</t>
         </is>
       </c>
     </row>
@@ -1539,12 +1539,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Best Drip Coffee Makers of 2026, Tested by Experts</t>
+          <t>Best Decking of 2026, Tested by Experts</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/appliances/coffee-makers/best-drip-coffee-makers-consumer-reports-tests-a1869713908/</t>
+          <t>https://www.consumerreports.org/home-garden/decking/best-decking-materials-from-consumer-reports-tests-a6751297873/</t>
         </is>
       </c>
     </row>
@@ -1556,12 +1556,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Consumer Safety Agency Finalizes New Regulations on Water Beads and Infant Neck Floats</t>
+          <t>Best TV Brands of 2026</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/babies-kids/toys/consumer-safety-agency-new-rules-water-beads-neck-floats-a2051187866/</t>
+          <t>https://www.consumerreports.org/electronics-computers/tvs/best-tv-brands-a7582471181/</t>
         </is>
       </c>
     </row>
@@ -1573,12 +1573,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>7 Best Food Processors and Choppers of 2026, Lab-Tested and Reviewed</t>
+          <t>4 Best Toilet Brushes of 2026 From Our Evaluations</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/appliances/food-processors-choppers/best-food-processors-of-the-year-a7878155198/</t>
+          <t>https://www.consumerreports.org/home-garden/toilets/best-toilet-brushes-a6509646029/</t>
         </is>
       </c>
     </row>
@@ -1590,12 +1590,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>4 Best Whole-House Heat Pumps of 2026, Lab-Tested and Reviewed</t>
+          <t>11 Best Cordless Drills of 2026, Lab-Tested and Reviewed</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/appliances/heat-pumps/best-whole-house-heat-pumps-a1157154177/</t>
+          <t>https://www.consumerreports.org/home-garden/cordless-drills-impact-drivers/best-cordless-drills-of-the-year-a1168250583/</t>
         </is>
       </c>
     </row>
@@ -1607,12 +1607,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>10 Tips to Get the Most Out of a Tank of Gas</t>
+          <t>9 Best Stick Vacuums of 2026, Lab-Tested and Reviewed</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/cars/fuel-economy-efficiency/10-tips-to-get-the-most-out-of-a-tank-of-gas-a2642110189/</t>
+          <t>https://www.consumerreports.org/appliances/vacuum-cleaners/best-stick-vacuums-of-the-year-a1113185163/</t>
         </is>
       </c>
     </row>
@@ -1624,12 +1624,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Best Nail Clippers for Every Need and Every Nail</t>
+          <t>Best Deals on Health and Beauty Products</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/health/personal-care/best-nail-clippers-a6951655841/</t>
+          <t>https://www.consumerreports.org/money/sales-promotions/best-deals-on-health-and-beauty-products-a1654821936/</t>
         </is>
       </c>
     </row>
@@ -1641,12 +1641,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Talking Carts 11: Couponing 101</t>
+          <t>Best Washers for $800 or Less</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/money/shopping-retail/talking-carts-11-couponing-101-a9760148597/</t>
+          <t>https://www.consumerreports.org/appliances/washing-machines/best-washers-for-800-dollars-or-less-a3982320572/</t>
         </is>
       </c>
     </row>
@@ -1658,12 +1658,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Best New SUVs and Cars for Under $30,000</t>
+          <t>Best Deals on Vacuums</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/cars/best-new-cars-under-30000-dollars-a6574737993/</t>
+          <t>https://www.consumerreports.org/appliances/vacuum-cleaners/best-vacuum-deals-right-now-a5043984151/</t>
         </is>
       </c>
     </row>
@@ -1675,12 +1675,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Simple Ways to Organize Your Home's Entryway</t>
+          <t>Buying or Leasing a Car in 2026: Which Makes the Best Financial Sense for You?</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/home-garden/home-organization/easy-tips-to-organize-home-entryway-a1146889912/</t>
+          <t>https://www.consumerreports.org/cars/buying-a-car/leasing-vs-buying-a-new-car-a9135602164/</t>
         </is>
       </c>
     </row>
@@ -1692,12 +1692,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>How to Save Money at the Gas Pump</t>
+          <t>Popular Cars and SUVs to Avoid and Safer Choices to Buy Instead</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/money/saving-money/how-to-save-money-at-the-gas-pump-a8520505361/</t>
+          <t>https://www.consumerreports.org/cars/car-safety/popular-cars-suvs-to-avoid-safer-choices-to-buy-instead-a7755684192/</t>
         </is>
       </c>
     </row>
@@ -1709,12 +1709,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>9 Best Stick Vacuums of 2026, Lab-Tested and Reviewed</t>
+          <t>How to Save Money at the Gas Pump</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/appliances/vacuum-cleaners/best-stick-vacuums-of-the-year-a1113185163/</t>
+          <t>https://www.consumerreports.org/money/saving-money/how-to-save-money-at-the-gas-pump-a8520505361/</t>
         </is>
       </c>
     </row>
@@ -1726,12 +1726,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Popular Cars and SUVs to Avoid and Safer Choices to Buy Instead</t>
+          <t>Simple Ways to Organize Your Home's Entryway</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/cars/car-safety/popular-cars-suvs-to-avoid-safer-choices-to-buy-instead-a7755684192/</t>
+          <t>https://www.consumerreports.org/home-garden/home-organization/easy-tips-to-organize-home-entryway-a1146889912/</t>
         </is>
       </c>
     </row>
@@ -1743,12 +1743,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Buying or Leasing a Car in 2026: Which Makes the Best Financial Sense for You?</t>
+          <t>Best New SUVs and Cars for Under $30,000</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/cars/buying-a-car/leasing-vs-buying-a-new-car-a9135602164/</t>
+          <t>https://www.consumerreports.org/cars/best-new-cars-under-30000-dollars-a6574737993/</t>
         </is>
       </c>
     </row>
@@ -1760,12 +1760,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Best Deals on Vacuums</t>
+          <t>Talking Carts 11: Couponing 101</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/appliances/vacuum-cleaners/best-vacuum-deals-right-now-a5043984151/</t>
+          <t>https://www.consumerreports.org/money/shopping-retail/talking-carts-11-couponing-101-a9760148597/</t>
         </is>
       </c>
     </row>
@@ -1777,12 +1777,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Best Washers for $800 or Less</t>
+          <t>Best Nail Clippers for Every Need and Every Nail</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/appliances/washing-machines/best-washers-for-800-dollars-or-less-a3982320572/</t>
+          <t>https://www.consumerreports.org/health/personal-care/best-nail-clippers-a6951655841/</t>
         </is>
       </c>
     </row>
@@ -1794,12 +1794,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Best Deals on Health and Beauty Products</t>
+          <t>10 Tips to Get the Most Out of a Tank of Gas</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/money/sales-promotions/best-deals-on-health-and-beauty-products-a1654821936/</t>
+          <t>https://www.consumerreports.org/cars/fuel-economy-efficiency/10-tips-to-get-the-most-out-of-a-tank-of-gas-a2642110189/</t>
         </is>
       </c>
     </row>
@@ -1811,12 +1811,12 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Best Battery Platforms for Power Tools</t>
+          <t>4 Best Glass Cleaners From Our Evaluations</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/home-garden/battery-platforms/best-battery-platforms-for-power-tools-a1200820570/</t>
+          <t>https://www.consumerreports.org/home-garden/cleaning/best-glass-cleaners-a9011399777/</t>
         </is>
       </c>
     </row>
@@ -1828,12 +1828,12 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Preview: 2027 BMW i3 Returns as an All-Electric Sedan</t>
+          <t>Our Favorite Deals Right Now</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/cars/hybrids-evs/2027-bmw-i3-review-a6401226776/</t>
+          <t>https://www.consumerreports.org/money/sales-promotions/our-favorite-deals-a4347518393/</t>
         </is>
       </c>
     </row>
@@ -1845,12 +1845,12 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>8 Midsized Three-Row Sport-Utility Vehicles With the Best Tested Gas Mileage</t>
+          <t>16 Best Washing Machines of 2026, Lab-Tested and Reviewed</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/cars/suvs/most-fuel-efficient-used-three-row-suvs-a7976679803/</t>
+          <t>https://www.consumerreports.org/appliances/washing-machines/best-washing-machines-of-the-year-a7327583525/</t>
         </is>
       </c>
     </row>
@@ -1862,12 +1862,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Best Cleaning Products From Our Tests and Evaluations</t>
+          <t>Best Deals on Tech Products Right Now</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/home-garden/cleaning/best-cleaning-products-a3675714062/</t>
+          <t>https://www.consumerreports.org/money/sales-promotions/best-electronics-deals-right-now-a3598707304/</t>
         </is>
       </c>
     </row>
@@ -1879,12 +1879,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Talking Cars 498: Discussing the Latest Electric Car Range Test Results</t>
+          <t>Best Mattress Sales Right Now</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/cars/cars-driving/talking-cars-498-latest-electric-car-range-test-results-a4872039008/</t>
+          <t>https://www.consumerreports.org/home-garden/mattresses/best-mattress-deals-a6347099135/</t>
         </is>
       </c>
     </row>
@@ -1896,12 +1896,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>4 Best Glass Cleaners From Our Evaluations</t>
+          <t>Talking Cars 498: Discussing the Latest Electric Car Range Test Results</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/home-garden/cleaning/best-glass-cleaners-a9011399777/</t>
+          <t>https://www.consumerreports.org/cars/cars-driving/talking-cars-498-latest-electric-car-range-test-results-a4872039008/</t>
         </is>
       </c>
     </row>
@@ -1913,12 +1913,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Best Deals on Tech Products Right Now</t>
+          <t>Preview: 2027 BMW i3 Returns as an All-Electric Sedan</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/money/sales-promotions/best-electronics-deals-right-now-a3598707304/</t>
+          <t>https://www.consumerreports.org/cars/hybrids-evs/2027-bmw-i3-review-a6401226776/</t>
         </is>
       </c>
     </row>
@@ -1930,12 +1930,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>16 Best Washing Machines of 2026, Lab-Tested and Reviewed</t>
+          <t>Best Battery Platforms for Power Tools</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/appliances/washing-machines/best-washing-machines-of-the-year-a7327583525/</t>
+          <t>https://www.consumerreports.org/home-garden/battery-platforms/best-battery-platforms-for-power-tools-a1200820570/</t>
         </is>
       </c>
     </row>
@@ -1947,12 +1947,12 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Best Mattress Sales Right Now</t>
+          <t>Best Cleaning Products From Our Tests and Evaluations</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/home-garden/mattresses/best-mattress-deals-a6347099135/</t>
+          <t>https://www.consumerreports.org/home-garden/cleaning/best-cleaning-products-a3675714062/</t>
         </is>
       </c>
     </row>
@@ -1964,12 +1964,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Our Favorite Deals Right Now</t>
+          <t>8 Midsized Three-Row Sport-Utility Vehicles With the Best Tested Gas Mileage</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/money/sales-promotions/our-favorite-deals-a4347518393/</t>
+          <t>https://www.consumerreports.org/cars/suvs/most-fuel-efficient-used-three-row-suvs-a7976679803/</t>
         </is>
       </c>
     </row>
@@ -1981,12 +1981,12 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Best Deals on Pet Products</t>
+          <t>Best Cars, SUVs, and Trucks from American Brands</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/money/discounts-rebates/best-deals-on-pet-products-a5737541283/</t>
+          <t>https://www.consumerreports.org/cars/cars-best-american-cars-suvs-trucks-a1034107548/</t>
         </is>
       </c>
     </row>
@@ -1998,12 +1998,12 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Best Cars, SUVs, and Trucks from American Brands</t>
+          <t>Raw Farm Raw Milk Cheddar Cheese Linked to an E. Coli Outbreak</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/cars/cars-best-american-cars-suvs-trucks-a1034107548/</t>
+          <t>https://www.consumerreports.org/health/food-recalls/raw-farm-raw-milk-cheddar-cheese-e-coli-outbreak-a1754162551/</t>
         </is>
       </c>
     </row>
@@ -2015,12 +2015,12 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Raw Farm Raw Milk Cheddar Cheese Linked to an E. Coli Outbreak</t>
+          <t>Worst Vacuums We Tested—and What to Buy Instead</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/health/food-recalls/raw-farm-raw-milk-cheddar-cheese-e-coli-outbreak-a1754162551/</t>
+          <t>https://www.consumerreports.org/appliances/vacuum-cleaners/worst-vacuums-we-tested-and-what-to-buy-instead-a4744433209/</t>
         </is>
       </c>
     </row>
@@ -2032,12 +2032,12 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Worst Vacuums We Tested—and What to Buy Instead</t>
+          <t>Best Hot Combs, Tested and Reviewed</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/appliances/vacuum-cleaners/worst-vacuums-we-tested-and-what-to-buy-instead-a4744433209/</t>
+          <t>https://www.consumerreports.org/health/hair-styling-tools/best-hot-combs-a1155859440/</t>
         </is>
       </c>
     </row>
@@ -2049,12 +2049,12 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Best Hot Combs, Tested and Reviewed</t>
+          <t>42 Used Cars to Avoid Buying</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/health/hair-styling-tools/best-hot-combs-a1155859440/</t>
+          <t>https://www.consumerreports.org/cars/used-cars-to-avoid-buying-a4034931071/</t>
         </is>
       </c>
     </row>
@@ -2066,12 +2066,12 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>42 Used Cars to Avoid Buying</t>
+          <t>Most Fuel-Efficient Used Hybrid Cars and Hatchbacks</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/cars/used-cars-to-avoid-buying-a4034931071/</t>
+          <t>https://www.consumerreports.org/cars/hybrids-evs/used-hybrid-sedans-and-hatchbacks-with-best-fuel-economy-a2840918797/</t>
         </is>
       </c>
     </row>
@@ -2083,12 +2083,12 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Most Fuel-Efficient Used Hybrid Cars and Hatchbacks</t>
+          <t>Least Durable Nonstick Frying Pans and What to Buy Instead</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/cars/hybrids-evs/used-hybrid-sedans-and-hatchbacks-with-best-fuel-economy-a2840918797/</t>
+          <t>https://www.consumerreports.org/home-garden/cookware/least-durable-nonstick-frying-pans-what-to-buy-instead-a4466494459/</t>
         </is>
       </c>
     </row>
@@ -2100,12 +2100,12 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Least Durable Nonstick Frying Pans and What to Buy Instead</t>
+          <t>How an Old-School Flip Phone Changed My Life</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/home-garden/cookware/least-durable-nonstick-frying-pans-what-to-buy-instead-a4466494459/</t>
+          <t>https://www.consumerreports.org/electronics-computers/cell-phones/pros-and-cons-of-using-a-flip-phone-a8412704280/</t>
         </is>
       </c>
     </row>
@@ -2117,12 +2117,12 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>How an Old-School Flip Phone Changed My Life</t>
+          <t>Best Deals on Pet Products</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/electronics-computers/cell-phones/pros-and-cons-of-using-a-flip-phone-a8412704280/</t>
+          <t>https://www.consumerreports.org/money/discounts-rebates/best-deals-on-pet-products-a5737541283/</t>
         </is>
       </c>
     </row>
@@ -2134,12 +2134,12 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Hyundai Recalls Palisade and Issues Stop-Sale After Child’s Death</t>
+          <t>Best Baby Food Companies for Reporting Lead, Arsenic, and Other Toxic Elements</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/cars/car-recalls-defects/hyundai-palisade-recall-folding-seats-stop-sale-child-death-a6861032164/</t>
+          <t>https://www.consumerreports.org/babies-kids/baby-food/baby-food-labels-heavy-metals-california-ab899-a5779555429/</t>
         </is>
       </c>
     </row>
@@ -2151,12 +2151,12 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>ICYMI: Spring Yard Prep, Exclusive Member Savings, Apple's New MacBook Neo</t>
+          <t>Consumer Reports’ Real-World Electric Car Range Comparison</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/home-garden/spring-yard-prep-exclusive-member-savings-apple-macbook-neo-a6548509942/</t>
+          <t>https://www.consumerreports.org/cars/hybrids-evs/real-world-ev-range-tests-models-that-beat-epa-estimates-a1103288135/</t>
         </is>
       </c>
     </row>
@@ -2168,12 +2168,12 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>7 Expert Steps to Buy a Used Car Without Costly Regrets</t>
+          <t>Best Spring Cleaning Deals on Vacuums, Carpet Cleaners, and More</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/cars/buying-a-car/how-to-protect-yourself-when-buying-a-used-car-a7040550851/</t>
+          <t>https://www.consumerreports.org/money/sales-promotions/best-spring-cleaning-deals-a6459257616/</t>
         </is>
       </c>
     </row>
@@ -2185,12 +2185,12 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Best Baby Food Companies for Reporting Lead, Arsenic, and Other Toxic Elements</t>
+          <t>7 Expert Steps to Buy a Used Car Without Costly Regrets</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/babies-kids/baby-food/baby-food-labels-heavy-metals-california-ab899-a5779555429/</t>
+          <t>https://www.consumerreports.org/cars/buying-a-car/how-to-protect-yourself-when-buying-a-used-car-a7040550851/</t>
         </is>
       </c>
     </row>
@@ -2202,12 +2202,12 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Best Spring Cleaning Deals on Vacuums, Carpet Cleaners, and More</t>
+          <t>ICYMI: Spring Yard Prep, Exclusive Member Savings, Apple's New MacBook Neo</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/money/sales-promotions/best-spring-cleaning-deals-a6459257616/</t>
+          <t>https://www.consumerreports.org/home-garden/spring-yard-prep-exclusive-member-savings-apple-macbook-neo-a6548509942/</t>
         </is>
       </c>
     </row>
@@ -2219,12 +2219,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Consumer Reports’ Real-World Electric Car Range Comparison</t>
+          <t>Hyundai Recalls Palisade and Issues Stop-Sale After Child’s Death</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/cars/hybrids-evs/real-world-ev-range-tests-models-that-beat-epa-estimates-a1103288135/</t>
+          <t>https://www.consumerreports.org/cars/car-recalls-defects/hyundai-palisade-recall-folding-seats-stop-sale-child-death-a6861032164/</t>
         </is>
       </c>
     </row>
@@ -2304,12 +2304,12 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>10 Best Deals on Electric Vehicles</t>
+          <t>Best Deals Under $50</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/cars/hybrids-evs/best-deals-on-electric-vehicles-a1198228201/</t>
+          <t>https://www.consumerreports.org/money/sales-promotions/best-deals-under-50-dollars-a2569975133/</t>
         </is>
       </c>
     </row>
@@ -2321,12 +2321,12 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>How to Stain a Deck</t>
+          <t>Best Deals Under $100</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/home-garden/wood-stains/how-to-stain-your-deck-a1462288683/</t>
+          <t>https://www.consumerreports.org/money/sales-promotions/best-deals-under-100-dollars-a1055650279/</t>
         </is>
       </c>
     </row>
@@ -2338,12 +2338,12 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Best Hybrid Cars for Under $35,000</t>
+          <t>4 Best K-Cup Coffee Makers of 2026, Lab-Tested and Reviewed</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/cars/fuel-economy-efficiency/best-hybrid-cars-from-consumer-reports-tests-a5841270718/</t>
+          <t>https://www.consumerreports.org/appliances/coffee-makers/best-keurig-k-cup-coffee-makers-a2682700597/</t>
         </is>
       </c>
     </row>
@@ -2355,12 +2355,12 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>20 Most Reliable and Fuel-Efficient 2026 Compact SUVs</t>
+          <t>5 Best Air Purifiers for Wildfire Smoke, According to Our Testing</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/cars/suvs/reliable-and-fuel-efficient-compact-suvs-a6901123061/</t>
+          <t>https://www.consumerreports.org/appliances/air-purifiers/best-air-purifiers-for-wildfire-smoke-a1153295134/</t>
         </is>
       </c>
     </row>
@@ -2372,12 +2372,12 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Toyota Highlander Recalled to Fix Second-Row Seat Latches</t>
+          <t>Does an ‘Eco-Friendly’ Diaper Really Exist?</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/cars/car-recalls-defects/toyota-highlander-recalled-to-fix-second-row-seat-latches-a1110263947/</t>
+          <t>https://www.consumerreports.org/babies-kids/diapers/does-an-eco-friendly-diaper-really-exist-a6768931967/</t>
         </is>
       </c>
     </row>
@@ -2389,12 +2389,12 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Best Deals Under $50</t>
+          <t>Toyota Highlander Recalled to Fix Second-Row Seat Latches</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/money/sales-promotions/best-deals-under-50-dollars-a2569975133/</t>
+          <t>https://www.consumerreports.org/cars/car-recalls-defects/toyota-highlander-recalled-to-fix-second-row-seat-latches-a1110263947/</t>
         </is>
       </c>
     </row>
@@ -2406,12 +2406,12 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Does an ‘Eco-Friendly’ Diaper Really Exist?</t>
+          <t>20 Most Reliable and Fuel-Efficient 2026 Compact SUVs</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/babies-kids/diapers/does-an-eco-friendly-diaper-really-exist-a6768931967/</t>
+          <t>https://www.consumerreports.org/cars/suvs/reliable-and-fuel-efficient-compact-suvs-a6901123061/</t>
         </is>
       </c>
     </row>
@@ -2423,12 +2423,12 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>5 Best Air Purifiers for Wildfire Smoke, According to Our Testing</t>
+          <t>How to Stain a Deck</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/appliances/air-purifiers/best-air-purifiers-for-wildfire-smoke-a1153295134/</t>
+          <t>https://www.consumerreports.org/home-garden/wood-stains/how-to-stain-your-deck-a1462288683/</t>
         </is>
       </c>
     </row>
@@ -2440,12 +2440,12 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>4 Best K-Cup Coffee Makers of 2026, Lab-Tested and Reviewed</t>
+          <t>10 Best Deals on Electric Vehicles</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/appliances/coffee-makers/best-keurig-k-cup-coffee-makers-a2682700597/</t>
+          <t>https://www.consumerreports.org/cars/hybrids-evs/best-deals-on-electric-vehicles-a1198228201/</t>
         </is>
       </c>
     </row>
@@ -2457,12 +2457,12 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Best Deals Under $100</t>
+          <t>Best Hybrid Cars for Under $35,000</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/money/sales-promotions/best-deals-under-100-dollars-a1055650279/</t>
+          <t>https://www.consumerreports.org/cars/fuel-economy-efficiency/best-hybrid-cars-from-consumer-reports-tests-a5841270718/</t>
         </is>
       </c>
     </row>
@@ -2474,12 +2474,12 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Best Used SUVs With Standout Fuel Economy</t>
+          <t>10 Cheap Cars That Consumer Reports Recommends</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/cars/suvs/most-fuel-efficient-5-year-old-compact-suvs-a1110308216/</t>
+          <t>https://www.consumerreports.org/cars/cheap-cars-recommended-by-consumer-reports-a1059266229/</t>
         </is>
       </c>
     </row>
@@ -2491,12 +2491,12 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Consumer Reports' Best Used Midsized SUVs With Excellent Fuel Economy</t>
+          <t>Most Discounted New Cars Right Now</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/cars/suvs/used-two-row-midsized-suvs-with-best-fuel-economy-a1177062626/</t>
+          <t>https://www.consumerreports.org/cars/buying-a-car/new-cars-with-biggest-savings-off-msrp-right-now-a1002706451/</t>
         </is>
       </c>
     </row>
@@ -2508,12 +2508,12 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Preview: 2026 Porsche Cayenne Electric Doesn’t Need to Plug In to Charge</t>
+          <t>Best Composite Decking of 2026, Tested by Experts</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/cars/suvs/2026-porsche-cayenne-electric-review-a1008258321/</t>
+          <t>https://www.consumerreports.org/home-garden/decking/best-composite-decking-from-consumer-reports-tests-a6753939440/</t>
         </is>
       </c>
     </row>
@@ -2525,12 +2525,12 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Best Deals on Healthy-Home Essentials</t>
+          <t>Worst Deals on New Cars Right Now</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/money/sales-promotions/best-deals-on-healthy-home-essentials-a5487006019/</t>
+          <t>https://www.consumerreports.org/cars/buying-a-car/worst-deals-on-new-cars-a3991316773/</t>
         </is>
       </c>
     </row>
@@ -2542,12 +2542,12 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>12 Products That Help Us Get a Good Night's Sleep</t>
+          <t>Most and Least Reliable Coffee Makers</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/health/sleeping/products-that-help-us-get-a-good-nights-sleep-a8894453489/</t>
+          <t>https://www.consumerreports.org/appliances/coffee-makers/most-and-least-reliable-coffee-makers-a4935369168/</t>
         </is>
       </c>
     </row>
@@ -2559,12 +2559,12 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Best Deals on Fitness Equipment and Accessories</t>
+          <t>Best and Worst Laundry Detergents of 2026</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/money/sales-promotions/best-deals-on-fitness-equipment-and-accessories-a9859972001/</t>
+          <t>https://www.consumerreports.org/appliances/laundry-detergents/best-and-worst-laundry-detergents-from-consumer-reports-tests-a9342715268/</t>
         </is>
       </c>
     </row>
@@ -2576,12 +2576,12 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>10 Cheap Cars That Consumer Reports Recommends</t>
+          <t>Best Deals on Smart Home Devices</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/cars/cheap-cars-recommended-by-consumer-reports-a1059266229/</t>
+          <t>https://www.consumerreports.org/home-garden/smart-home/best-smart-home-deals-a3525616797/</t>
         </is>
       </c>
     </row>
@@ -2593,12 +2593,12 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Best and Worst Laundry Detergents of 2026</t>
+          <t>Best Deals on Fitness Equipment and Accessories</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/appliances/laundry-detergents/best-and-worst-laundry-detergents-from-consumer-reports-tests-a9342715268/</t>
+          <t>https://www.consumerreports.org/money/sales-promotions/best-deals-on-fitness-equipment-and-accessories-a9859972001/</t>
         </is>
       </c>
     </row>
@@ -2610,12 +2610,12 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Most and Least Reliable Coffee Makers</t>
+          <t>Best Deals on Healthy-Home Essentials</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/appliances/coffee-makers/most-and-least-reliable-coffee-makers-a4935369168/</t>
+          <t>https://www.consumerreports.org/money/sales-promotions/best-deals-on-healthy-home-essentials-a5487006019/</t>
         </is>
       </c>
     </row>
@@ -2627,12 +2627,12 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Worst Deals on New Cars Right Now</t>
+          <t>Preview: 2026 Porsche Cayenne Electric Doesn’t Need to Plug In to Charge</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/cars/buying-a-car/worst-deals-on-new-cars-a3991316773/</t>
+          <t>https://www.consumerreports.org/cars/suvs/2026-porsche-cayenne-electric-review-a1008258321/</t>
         </is>
       </c>
     </row>
@@ -2644,12 +2644,12 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Best Composite Decking of 2026, Tested by Experts</t>
+          <t>Best Used SUVs With Standout Fuel Economy</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/home-garden/decking/best-composite-decking-from-consumer-reports-tests-a6753939440/</t>
+          <t>https://www.consumerreports.org/cars/suvs/most-fuel-efficient-5-year-old-compact-suvs-a1110308216/</t>
         </is>
       </c>
     </row>
@@ -2661,12 +2661,12 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Best Deals on Smart Home Devices</t>
+          <t>Consumer Reports' Best Used Midsized SUVs With Excellent Fuel Economy</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/home-garden/smart-home/best-smart-home-deals-a3525616797/</t>
+          <t>https://www.consumerreports.org/cars/suvs/used-two-row-midsized-suvs-with-best-fuel-economy-a1177062626/</t>
         </is>
       </c>
     </row>
@@ -2678,12 +2678,12 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Most Discounted New Cars Right Now</t>
+          <t>12 Products That Help Us Get a Good Night's Sleep</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/cars/buying-a-car/new-cars-with-biggest-savings-off-msrp-right-now-a1002706451/</t>
+          <t>https://www.consumerreports.org/health/sleeping/products-that-help-us-get-a-good-nights-sleep-a8894453489/</t>
         </is>
       </c>
     </row>
@@ -2695,12 +2695,12 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Best Deals on SUVs You Can Buy Right Now</t>
+          <t>Which iPhone Should You Buy?</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/cars/suvs/best-deals-on-new-suvs-a3535956359/</t>
+          <t>https://www.consumerreports.org/electronics-computers/cell-phones/which-iphone-should-you-buy-a7028071026/</t>
         </is>
       </c>
     </row>
@@ -2712,12 +2712,12 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Talking Cars 497: Should You Drive 55 to Save Gas?</t>
+          <t>Best Deals on Home Products</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/cars/cars-driving/talking-cars-497-should-you-drive-55-to-save-gas-a3968521620/</t>
+          <t>https://www.consumerreports.org/money/sales-promotions/best-deals-on-home-products-a1464868801/</t>
         </is>
       </c>
     </row>
@@ -2729,12 +2729,12 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Popular Small Cars to Avoid and What to Buy Instead</t>
+          <t>Best Deals on Kitchen Products</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/cars/buying-a-car/popular-compact-cars-to-avoid-what-to-buy-instead-a1188453224/</t>
+          <t>https://www.consumerreports.org/money/sales-promotions/best-deals-on-kitchen-products-a3665220041/</t>
         </is>
       </c>
     </row>
@@ -2746,12 +2746,12 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>How Do Hybrid Cars Work?</t>
+          <t>8 Best Coffee Makers of 2026, Lab Tested and Reviewed</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/cars/hybrids-evs/how-do-hybrid-cars-work-a1034181509/</t>
+          <t>https://www.consumerreports.org/appliances/coffee-makers/best-coffee-makers-of-the-year-a9612622702/</t>
         </is>
       </c>
     </row>
@@ -2763,12 +2763,12 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Best New-Car Deals</t>
+          <t>Best Deals on Fuel-Efficient Cars and SUVs</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/cars/best-new-car-deals-a1060496430/</t>
+          <t>https://www.consumerreports.org/cars/buying-a-car/best-deals-on-fuel-efficient-cars-a4329802409/</t>
         </is>
       </c>
     </row>
@@ -2780,12 +2780,12 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Which iPhone Should You Buy?</t>
+          <t>Best New-Car Deals</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/electronics-computers/cell-phones/which-iphone-should-you-buy-a7028071026/</t>
+          <t>https://www.consumerreports.org/cars/best-new-car-deals-a1060496430/</t>
         </is>
       </c>
     </row>
@@ -2797,12 +2797,12 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Best Deals on Fuel-Efficient Cars and SUVs</t>
+          <t>How Do Hybrid Cars Work?</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/cars/buying-a-car/best-deals-on-fuel-efficient-cars-a4329802409/</t>
+          <t>https://www.consumerreports.org/cars/hybrids-evs/how-do-hybrid-cars-work-a1034181509/</t>
         </is>
       </c>
     </row>
@@ -2814,12 +2814,12 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>8 Best Coffee Makers of 2026, Lab Tested and Reviewed</t>
+          <t>Popular Small Cars to Avoid and What to Buy Instead</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/appliances/coffee-makers/best-coffee-makers-of-the-year-a9612622702/</t>
+          <t>https://www.consumerreports.org/cars/buying-a-car/popular-compact-cars-to-avoid-what-to-buy-instead-a1188453224/</t>
         </is>
       </c>
     </row>
@@ -2831,12 +2831,12 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Best Deals on Kitchen Products</t>
+          <t>Talking Cars 497: Should You Drive 55 to Save Gas?</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/money/sales-promotions/best-deals-on-kitchen-products-a3665220041/</t>
+          <t>https://www.consumerreports.org/cars/cars-driving/talking-cars-497-should-you-drive-55-to-save-gas-a3968521620/</t>
         </is>
       </c>
     </row>
@@ -2848,12 +2848,12 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Best Deals on Home Products</t>
+          <t>Best Deals on SUVs You Can Buy Right Now</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/money/sales-promotions/best-deals-on-home-products-a1464868801/</t>
+          <t>https://www.consumerreports.org/cars/suvs/best-deals-on-new-suvs-a3535956359/</t>
         </is>
       </c>
     </row>
@@ -2865,12 +2865,12 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>14 Exclusive Savings for CR's Member Appreciation Week</t>
+          <t>Best Sales on Pillows, Duvets, and More Sleep Essentials</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/money/shopping-retail/member-exclusive-savings-a4229795581/</t>
+          <t>https://www.consumerreports.org/money/sales-promotions/best-deals-on-pillows-sheets-and-other-sleep-accessories-a9893546733/</t>
         </is>
       </c>
     </row>
@@ -2882,12 +2882,12 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Best Cars Made in the USA</t>
+          <t>Consumer Reports' Cars With the Best Gas Mileage</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/cars/best-cars-made-in-the-usa-a7966845571/</t>
+          <t>https://www.consumerreports.org/cars/fuel-economy-efficiency/the-most-fuel-efficient-cars-best-mpg-a1198903400/</t>
         </is>
       </c>
     </row>
@@ -2899,12 +2899,12 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Safest Midsized, Large, and Three-Row SUVs of 2026</t>
+          <t>What's the Best Mac Laptop or Desktop for You?</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/cars/car-safety/safest-midsized-large-three-row-suvs-a4483160846/</t>
+          <t>https://www.consumerreports.org/electronics-computers/computers/best-mac-desktop-or-laptop-for-you-a1085516654/</t>
         </is>
       </c>
     </row>
@@ -2916,12 +2916,12 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>5 Best Umbrellas, Tested by Our Experts</t>
+          <t>Trader Joe's Chicken Fried Rice Recall Expanded. Packages May Contain Glass Fragments.</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/apparel-accessories/best-umbrellas-a5725351696/</t>
+          <t>https://www.consumerreports.org/health/food-recalls/fried-rice-ramen-dumpling-recall-glass-trader-joes-ajinomoto-a1204133892/</t>
         </is>
       </c>
     </row>
@@ -2933,12 +2933,12 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>What's the Best Mac Laptop or Desktop for You?</t>
+          <t>Safest Midsized, Large, and Three-Row SUVs of 2026</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/electronics-computers/computers/best-mac-desktop-or-laptop-for-you-a1085516654/</t>
+          <t>https://www.consumerreports.org/cars/car-safety/safest-midsized-large-three-row-suvs-a4483160846/</t>
         </is>
       </c>
     </row>
@@ -2950,12 +2950,12 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Trader Joe's Chicken Fried Rice Recall Expanded. Packages May Contain Glass Fragments.</t>
+          <t>5 Best Umbrellas, Tested by Our Experts</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/health/food-recalls/fried-rice-ramen-dumpling-recall-glass-trader-joes-ajinomoto-a1204133892/</t>
+          <t>https://www.consumerreports.org/apparel-accessories/best-umbrellas-a5725351696/</t>
         </is>
       </c>
     </row>
@@ -2967,12 +2967,12 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Consumer Reports' Cars With the Best Gas Mileage</t>
+          <t>14 Exclusive Savings for CR's Member Appreciation Week</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/cars/fuel-economy-efficiency/the-most-fuel-efficient-cars-best-mpg-a1198903400/</t>
+          <t>https://www.consumerreports.org/money/shopping-retail/member-exclusive-savings-a4229795581/</t>
         </is>
       </c>
     </row>
@@ -2984,12 +2984,12 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Best Sales on Pillows, Duvets, and More Sleep Essentials</t>
+          <t>Best Cars Made in the USA</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/money/sales-promotions/best-deals-on-pillows-sheets-and-other-sleep-accessories-a9893546733/</t>
+          <t>https://www.consumerreports.org/cars/best-cars-made-in-the-usa-a7966845571/</t>
         </is>
       </c>
     </row>
@@ -3171,12 +3171,12 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>How Do You Maintain a Car That Isn’t Driven Much?</t>
+          <t>6 Best Impact Drivers of 2026, Lab-Tested and Reviewed</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/cars/car-maintenance/how-to-maintain-a-car-that-isnt-driven-much-a6412749580/</t>
+          <t>https://www.consumerreports.org/home-garden/cordless-drills-impact-drivers/best-impact-drivers-of-the-year-a2626906980/</t>
         </is>
       </c>
     </row>
@@ -3188,12 +3188,12 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>6 Best Impact Drivers of 2026, Lab-Tested and Reviewed</t>
+          <t>How Do You Maintain a Car That Isn’t Driven Much?</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>https://www.consumerreports.org/home-garden/cordless-drills-impact-drivers/best-impact-drivers-of-the-year-a2626906980/</t>
+          <t>https://www.consumerreports.org/cars/car-maintenance/how-to-maintain-a-car-that-isnt-driven-much-a6412749580/</t>
         </is>
       </c>
     </row>

</xml_diff>